<commit_message>
Add supervisor field to profile, Escape cancels a loading export (v1.2.3)
- New "Your supervisor" field on the account page, printed under the
  "Approved By (Please Print)" label on the exported spreadsheet (cell F5,
  merged F5:H5 in the template - added per explicit request). New
  additive `supervisor` column on users, same pattern as employee_number/
  department, including the missing-info badge.
- Pressing Escape while a report export's loading overlay is showing now
  actually aborts the in-flight fetch instead of just leaving the overlay
  spinning with no way out. Extended showLoadingOverlay() with an optional
  cancel callback (Escape-to-cancel is opt-in per caller, since the upload
  flow's overlay wraps a real form submission that can't be aborted this
  way).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Expense_Report_General.xlsx
+++ b/templates/Expense_Report_General.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gascond\Desktop\GitHub\ExpenseReportService\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9FCCCC-F0C5-4C62-8F35-D59FA6E72B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A102FC1D-3E14-4B57-8DF2-12AD6DD2F13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -283,7 +283,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="44">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -806,11 +806,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -847,12 +867,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -1008,6 +1022,23 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1016,46 +1047,38 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1065,9 +1088,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" shrinkToFit="1"/>
       <protection locked="0"/>
@@ -1077,6 +1097,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1449,8 +1484,8 @@
     <col min="7" max="7" width="10.42578125" customWidth="1"/>
     <col min="8" max="8" width="10.140625" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="22.85546875" customWidth="1"/>
     <col min="13" max="13" width="9.28515625" customWidth="1"/>
   </cols>
@@ -1478,10 +1513,10 @@
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="92" t="s">
+      <c r="B2" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="92"/>
+      <c r="C2" s="99"/>
       <c r="D2" s="7" t="s">
         <v>4</v>
       </c>
@@ -1505,64 +1540,64 @@
     </row>
     <row r="3" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
-      <c r="D3" s="16">
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="75">
         <v>6288</v>
       </c>
-      <c r="E3" s="17">
+      <c r="E3" s="76">
         <v>46185</v>
       </c>
       <c r="F3" s="93" t="s">
         <v>9</v>
       </c>
       <c r="G3" s="93"/>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="19"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="18" t="s">
+      <c r="I3" s="17"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="19"/>
-      <c r="M3" s="21"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="19"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
       <c r="F4" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="24" t="s">
+      <c r="G4" s="74"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="26"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="24"/>
     </row>
     <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="31"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="96"/>
+      <c r="G5" s="97"/>
+      <c r="H5" s="98"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="29"/>
     </row>
     <row r="6" spans="1:13" ht="13.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="94" t="s">
@@ -1577,23 +1612,23 @@
       <c r="F6" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="89" t="s">
+      <c r="G6" s="90" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="89" t="s">
+      <c r="H6" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="89" t="s">
+      <c r="I6" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="89" t="s">
+      <c r="J6" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="89"/>
-      <c r="L6" s="90" t="s">
+      <c r="K6" s="90"/>
+      <c r="L6" s="91" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="91" t="s">
+      <c r="M6" s="92" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1604,13 +1639,13 @@
       <c r="D7" s="95"/>
       <c r="E7" s="95"/>
       <c r="F7" s="95"/>
-      <c r="G7" s="89"/>
-      <c r="H7" s="89"/>
-      <c r="I7" s="89"/>
-      <c r="J7" s="89"/>
-      <c r="K7" s="89"/>
-      <c r="L7" s="90"/>
-      <c r="M7" s="91"/>
+      <c r="G7" s="90"/>
+      <c r="H7" s="90"/>
+      <c r="I7" s="90"/>
+      <c r="J7" s="90"/>
+      <c r="K7" s="90"/>
+      <c r="L7" s="91"/>
+      <c r="M7" s="92"/>
     </row>
     <row r="8" spans="1:13" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="94"/>
@@ -1619,13 +1654,13 @@
       <c r="D8" s="95"/>
       <c r="E8" s="95"/>
       <c r="F8" s="95"/>
-      <c r="G8" s="89"/>
-      <c r="H8" s="89"/>
-      <c r="I8" s="89"/>
-      <c r="J8" s="89"/>
-      <c r="K8" s="89"/>
-      <c r="L8" s="90"/>
-      <c r="M8" s="91"/>
+      <c r="G8" s="90"/>
+      <c r="H8" s="90"/>
+      <c r="I8" s="90"/>
+      <c r="J8" s="90"/>
+      <c r="K8" s="90"/>
+      <c r="L8" s="91"/>
+      <c r="M8" s="92"/>
     </row>
     <row r="9" spans="1:13" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="94"/>
@@ -1634,250 +1669,250 @@
       <c r="D9" s="95"/>
       <c r="E9" s="95"/>
       <c r="F9" s="95"/>
-      <c r="G9" s="89"/>
-      <c r="H9" s="89"/>
-      <c r="I9" s="89"/>
-      <c r="J9" s="89"/>
-      <c r="K9" s="89"/>
-      <c r="L9" s="90"/>
-      <c r="M9" s="91"/>
+      <c r="G9" s="90"/>
+      <c r="H9" s="90"/>
+      <c r="I9" s="90"/>
+      <c r="J9" s="90"/>
+      <c r="K9" s="90"/>
+      <c r="L9" s="91"/>
+      <c r="M9" s="92"/>
     </row>
     <row r="10" spans="1:13" ht="27" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="72">
+      <c r="A10" s="70">
         <v>46094.482615740701</v>
       </c>
-      <c r="B10" s="87" t="s">
+      <c r="B10" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="87"/>
-      <c r="D10" s="87"/>
-      <c r="E10" s="87"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34">
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32">
         <v>239.98</v>
       </c>
       <c r="J10" s="82"/>
       <c r="K10" s="83"/>
-      <c r="L10" s="35" t="s">
+      <c r="L10" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="M10" s="36">
+      <c r="M10" s="34">
         <f t="shared" ref="M10:M35" si="0">IF(SUM(F10:K10)&gt;0,SUM(F10:K10),"")</f>
         <v>239.98</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="72">
+      <c r="A11" s="70">
         <v>46119.330486111103</v>
       </c>
-      <c r="B11" s="87" t="s">
+      <c r="B11" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="87"/>
-      <c r="D11" s="87"/>
-      <c r="E11" s="87"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="33">
+      <c r="C11" s="86"/>
+      <c r="D11" s="86"/>
+      <c r="E11" s="86"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="31">
         <v>35.1</v>
       </c>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="77"/>
-      <c r="L11" s="35" t="s">
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="79"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="M11" s="36">
+      <c r="M11" s="34">
         <f t="shared" si="0"/>
         <v>35.1</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="72">
+      <c r="A12" s="70">
         <v>46129.313067129602</v>
       </c>
-      <c r="B12" s="87" t="s">
+      <c r="B12" s="86" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="87"/>
-      <c r="D12" s="87"/>
-      <c r="E12" s="87"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="33">
+      <c r="C12" s="86"/>
+      <c r="D12" s="86"/>
+      <c r="E12" s="86"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="31">
         <v>28.98</v>
       </c>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="76"/>
-      <c r="K12" s="77"/>
-      <c r="L12" s="35" t="s">
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="79"/>
+      <c r="K12" s="80"/>
+      <c r="L12" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="36">
+      <c r="M12" s="34">
         <f t="shared" si="0"/>
         <v>28.98</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="72">
+      <c r="A13" s="70">
         <v>46132.458703703698</v>
       </c>
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="87"/>
-      <c r="D13" s="87"/>
-      <c r="E13" s="87"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33">
+      <c r="C13" s="86"/>
+      <c r="D13" s="86"/>
+      <c r="E13" s="86"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="31">
         <v>34.880000000000003</v>
       </c>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="76"/>
-      <c r="K13" s="77"/>
-      <c r="L13" s="35" t="s">
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="80"/>
+      <c r="L13" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="M13" s="36">
+      <c r="M13" s="34">
         <f t="shared" si="0"/>
         <v>34.880000000000003</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="72">
+      <c r="A14" s="70">
         <v>46132.512962963003</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="86" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="87"/>
-      <c r="D14" s="87"/>
-      <c r="E14" s="87"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="33">
+      <c r="C14" s="86"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="31">
         <v>24.99</v>
       </c>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="76"/>
-      <c r="K14" s="77"/>
-      <c r="L14" s="35" t="s">
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="80"/>
+      <c r="L14" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="M14" s="36">
+      <c r="M14" s="34">
         <f t="shared" si="0"/>
         <v>24.99</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="72">
+      <c r="A15" s="70">
         <v>46133.5090277778</v>
       </c>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="87"/>
-      <c r="D15" s="87"/>
-      <c r="E15" s="87"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33">
+      <c r="C15" s="86"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="86"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="31">
         <v>60.95</v>
       </c>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="76"/>
-      <c r="K15" s="77"/>
-      <c r="L15" s="35" t="s">
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="79"/>
+      <c r="K15" s="80"/>
+      <c r="L15" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="36">
+      <c r="M15" s="34">
         <f t="shared" si="0"/>
         <v>60.95</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="72">
+      <c r="A16" s="70">
         <v>46149.514965277798</v>
       </c>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="86" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="87"/>
-      <c r="D16" s="87"/>
-      <c r="E16" s="87"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="33">
+      <c r="C16" s="86"/>
+      <c r="D16" s="86"/>
+      <c r="E16" s="86"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="31">
         <v>60.63</v>
       </c>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="76"/>
-      <c r="K16" s="77"/>
-      <c r="L16" s="35" t="s">
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="79"/>
+      <c r="K16" s="80"/>
+      <c r="L16" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="M16" s="36">
+      <c r="M16" s="34">
         <f t="shared" si="0"/>
         <v>60.63</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="72">
+      <c r="A17" s="70">
         <v>46156.383773148198</v>
       </c>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="87"/>
-      <c r="D17" s="87"/>
-      <c r="E17" s="87"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33">
+      <c r="C17" s="86"/>
+      <c r="D17" s="86"/>
+      <c r="E17" s="86"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="31">
         <v>54.9</v>
       </c>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="76"/>
-      <c r="K17" s="77"/>
-      <c r="L17" s="35" t="s">
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="79"/>
+      <c r="K17" s="80"/>
+      <c r="L17" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="M17" s="36">
+      <c r="M17" s="34">
         <f t="shared" si="0"/>
         <v>54.9</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="72">
+      <c r="A18" s="70">
         <v>46181.498541666697</v>
       </c>
-      <c r="B18" s="87" t="s">
+      <c r="B18" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="87"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="87"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33">
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="31">
         <v>56.92</v>
       </c>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="76"/>
-      <c r="K18" s="77"/>
-      <c r="L18" s="35" t="s">
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="79"/>
+      <c r="K18" s="80"/>
+      <c r="L18" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="M18" s="36">
+      <c r="M18" s="34">
         <f t="shared" si="0"/>
         <v>56.92</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="72">
+      <c r="A19" s="70">
         <v>46183.4688888889</v>
       </c>
       <c r="B19" s="88" t="s">
@@ -1886,306 +1921,306 @@
       <c r="C19" s="88"/>
       <c r="D19" s="88"/>
       <c r="E19" s="88"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="33">
+      <c r="F19" s="30"/>
+      <c r="G19" s="31">
         <v>36</v>
       </c>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="76"/>
-      <c r="K19" s="77"/>
-      <c r="L19" s="35" t="s">
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="79"/>
+      <c r="K19" s="80"/>
+      <c r="L19" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="M19" s="36">
+      <c r="M19" s="34">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="72"/>
-      <c r="B20" s="86"/>
-      <c r="C20" s="86"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="86"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="76"/>
-      <c r="K20" s="77"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="36" t="str">
+      <c r="A20" s="70"/>
+      <c r="B20" s="89"/>
+      <c r="C20" s="89"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="79"/>
+      <c r="K20" s="80"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="72"/>
-      <c r="B21" s="87"/>
-      <c r="C21" s="87"/>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="76"/>
-      <c r="K21" s="77"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="36" t="str">
+      <c r="A21" s="70"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="86"/>
+      <c r="D21" s="86"/>
+      <c r="E21" s="86"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="79"/>
+      <c r="K21" s="80"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="72"/>
-      <c r="B22" s="87"/>
-      <c r="C22" s="87"/>
-      <c r="D22" s="87"/>
-      <c r="E22" s="87"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="76"/>
-      <c r="K22" s="77"/>
-      <c r="L22" s="35"/>
-      <c r="M22" s="36" t="str">
+      <c r="A22" s="70"/>
+      <c r="B22" s="86"/>
+      <c r="C22" s="86"/>
+      <c r="D22" s="86"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="80"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="72"/>
-      <c r="B23" s="87"/>
-      <c r="C23" s="87"/>
-      <c r="D23" s="87"/>
-      <c r="E23" s="87"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="76"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="35"/>
-      <c r="M23" s="36" t="str">
+      <c r="A23" s="70"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="79"/>
+      <c r="K23" s="80"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="72"/>
-      <c r="B24" s="87"/>
-      <c r="C24" s="87"/>
-      <c r="D24" s="87"/>
-      <c r="E24" s="87"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="76"/>
-      <c r="K24" s="77"/>
-      <c r="L24" s="35"/>
-      <c r="M24" s="36" t="str">
+      <c r="A24" s="70"/>
+      <c r="B24" s="86"/>
+      <c r="C24" s="86"/>
+      <c r="D24" s="86"/>
+      <c r="E24" s="86"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="79"/>
+      <c r="K24" s="80"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="73"/>
-      <c r="B25" s="85"/>
-      <c r="C25" s="85"/>
-      <c r="D25" s="85"/>
-      <c r="E25" s="85"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="76"/>
-      <c r="K25" s="77"/>
-      <c r="L25" s="35"/>
-      <c r="M25" s="36" t="str">
+      <c r="A25" s="71"/>
+      <c r="B25" s="87"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="79"/>
+      <c r="K25" s="80"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="74"/>
+      <c r="A26" s="72"/>
       <c r="B26" s="84"/>
       <c r="C26" s="84"/>
       <c r="D26" s="84"/>
       <c r="E26" s="84"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="76"/>
-      <c r="K26" s="77"/>
-      <c r="L26" s="35"/>
-      <c r="M26" s="36" t="str">
+      <c r="F26" s="35"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="79"/>
+      <c r="K26" s="80"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="74"/>
+      <c r="A27" s="72"/>
       <c r="B27" s="84"/>
       <c r="C27" s="84"/>
       <c r="D27" s="84"/>
       <c r="E27" s="84"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="76"/>
-      <c r="K27" s="77"/>
-      <c r="L27" s="35"/>
-      <c r="M27" s="36" t="str">
+      <c r="F27" s="35"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="79"/>
+      <c r="K27" s="80"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="74"/>
+      <c r="A28" s="72"/>
       <c r="B28" s="84"/>
       <c r="C28" s="84"/>
       <c r="D28" s="84"/>
       <c r="E28" s="84"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="76"/>
-      <c r="K28" s="77"/>
-      <c r="L28" s="35"/>
-      <c r="M28" s="36" t="str">
+      <c r="F28" s="35"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="80"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="74"/>
+      <c r="A29" s="72"/>
       <c r="B29" s="84"/>
       <c r="C29" s="84"/>
       <c r="D29" s="84"/>
       <c r="E29" s="84"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="76"/>
-      <c r="K29" s="77"/>
-      <c r="L29" s="35"/>
-      <c r="M29" s="36" t="str">
+      <c r="F29" s="35"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="80"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="74"/>
+      <c r="A30" s="72"/>
       <c r="B30" s="84"/>
       <c r="C30" s="84"/>
       <c r="D30" s="84"/>
       <c r="E30" s="84"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="76"/>
-      <c r="K30" s="77"/>
-      <c r="L30" s="35"/>
-      <c r="M30" s="36" t="str">
+      <c r="F30" s="35"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="79"/>
+      <c r="K30" s="80"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A31" s="74"/>
+      <c r="A31" s="72"/>
       <c r="B31" s="84"/>
       <c r="C31" s="84"/>
       <c r="D31" s="84"/>
       <c r="E31" s="84"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="76"/>
-      <c r="K31" s="77"/>
-      <c r="L31" s="35"/>
-      <c r="M31" s="36" t="str">
+      <c r="F31" s="35"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="79"/>
+      <c r="K31" s="80"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="74"/>
+      <c r="A32" s="72"/>
       <c r="B32" s="84"/>
       <c r="C32" s="84"/>
       <c r="D32" s="84"/>
       <c r="E32" s="84"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="76"/>
-      <c r="K32" s="77"/>
-      <c r="L32" s="35"/>
-      <c r="M32" s="36" t="str">
+      <c r="F32" s="35"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="79"/>
+      <c r="K32" s="80"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A33" s="74"/>
+      <c r="A33" s="72"/>
       <c r="B33" s="84"/>
       <c r="C33" s="84"/>
       <c r="D33" s="84"/>
       <c r="E33" s="84"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="76"/>
-      <c r="K33" s="77"/>
-      <c r="L33" s="35"/>
-      <c r="M33" s="36" t="str">
+      <c r="F33" s="35"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="79"/>
+      <c r="K33" s="80"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A34" s="74"/>
+      <c r="A34" s="72"/>
       <c r="B34" s="84"/>
       <c r="C34" s="84"/>
       <c r="D34" s="84"/>
       <c r="E34" s="84"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
-      <c r="J34" s="76"/>
-      <c r="K34" s="77"/>
-      <c r="L34" s="35"/>
-      <c r="M34" s="36" t="str">
+      <c r="F34" s="35"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="79"/>
+      <c r="K34" s="80"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="75"/>
-      <c r="B35" s="80"/>
-      <c r="C35" s="80"/>
-      <c r="D35" s="80"/>
-      <c r="E35" s="80"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39"/>
-      <c r="J35" s="78"/>
-      <c r="K35" s="79"/>
-      <c r="L35" s="40"/>
-      <c r="M35" s="36" t="str">
+      <c r="A35" s="73"/>
+      <c r="B35" s="85"/>
+      <c r="C35" s="85"/>
+      <c r="D35" s="85"/>
+      <c r="E35" s="85"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="77"/>
+      <c r="K35" s="78"/>
+      <c r="L35" s="38"/>
+      <c r="M35" s="34" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -2198,145 +2233,146 @@
       <c r="C36" s="81"/>
       <c r="D36" s="81"/>
       <c r="E36" s="81"/>
-      <c r="F36" s="41" t="str">
+      <c r="F36" s="39" t="str">
         <f t="shared" ref="F36:K36" si="1">IF(SUM(F8:F35)&gt;0,SUM(F8:F35),"")</f>
         <v/>
       </c>
-      <c r="G36" s="41">
+      <c r="G36" s="39">
         <f t="shared" si="1"/>
         <v>393.35</v>
       </c>
-      <c r="H36" s="41" t="str">
+      <c r="H36" s="39" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I36" s="41">
+      <c r="I36" s="39">
         <f t="shared" si="1"/>
         <v>239.98</v>
       </c>
-      <c r="J36" s="42" t="str">
+      <c r="J36" s="40" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K36" s="43" t="str">
+      <c r="K36" s="41" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L36" s="41"/>
-      <c r="M36" s="44">
+      <c r="L36" s="39"/>
+      <c r="M36" s="42">
         <f>IF(SUM(M8:M35)=SUM(F36:K36),SUM(M8:M35),0)</f>
         <v>633.32999999999993</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A37" s="45"/>
-      <c r="B37" s="46" t="s">
+      <c r="A37" s="43"/>
+      <c r="B37" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="C37" s="46" t="s">
+      <c r="C37" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="D37" s="23"/>
-      <c r="E37" s="47"/>
-      <c r="F37" s="48" t="s">
+      <c r="D37" s="21"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="G37" s="49"/>
-      <c r="H37" s="50" t="s">
+      <c r="G37" s="47"/>
+      <c r="H37" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="I37" s="47"/>
-      <c r="J37" s="47"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="51"/>
-      <c r="M37" s="52"/>
+      <c r="I37" s="45"/>
+      <c r="J37" s="45"/>
+      <c r="K37" s="47"/>
+      <c r="L37" s="49"/>
+      <c r="M37" s="50"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A38" s="53" t="s">
+      <c r="A38" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="46" t="s">
+      <c r="B38" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="C38" s="54">
+      <c r="C38" s="52">
         <v>100</v>
       </c>
-      <c r="D38" s="55" t="s">
+      <c r="D38" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="E38" s="47"/>
-      <c r="F38" s="56" t="s">
+      <c r="E38" s="45"/>
+      <c r="F38" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="G38" s="51"/>
-      <c r="H38" s="51" t="s">
+      <c r="G38" s="49"/>
+      <c r="H38" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="51"/>
-      <c r="L38" s="51"/>
-      <c r="M38" s="57"/>
+      <c r="I38" s="45"/>
+      <c r="J38" s="45"/>
+      <c r="K38" s="49"/>
+      <c r="L38" s="49"/>
+      <c r="M38" s="55"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A39" s="58"/>
-      <c r="B39" s="59" t="s">
+      <c r="A39" s="56"/>
+      <c r="B39" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="60">
+      <c r="C39" s="58">
         <v>50</v>
       </c>
-      <c r="D39" s="61" t="s">
+      <c r="D39" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="E39" s="47"/>
-      <c r="F39" s="48" t="s">
+      <c r="E39" s="45"/>
+      <c r="F39" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="G39" s="51"/>
-      <c r="H39" s="51" t="s">
+      <c r="G39" s="49"/>
+      <c r="H39" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="51"/>
-      <c r="L39" s="51"/>
-      <c r="M39" s="57"/>
+      <c r="I39" s="45"/>
+      <c r="J39" s="45"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="49"/>
+      <c r="M39" s="55"/>
     </row>
     <row r="40" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="62"/>
-      <c r="B40" s="63" t="s">
+      <c r="A40" s="60"/>
+      <c r="B40" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="C40" s="64">
+      <c r="C40" s="62">
         <v>150</v>
       </c>
-      <c r="D40" s="65" t="s">
+      <c r="D40" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="E40" s="66"/>
-      <c r="F40" s="67" t="s">
+      <c r="E40" s="64"/>
+      <c r="F40" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="G40" s="68"/>
-      <c r="H40" s="69" t="s">
+      <c r="G40" s="66"/>
+      <c r="H40" s="67" t="s">
         <v>52</v>
       </c>
-      <c r="I40" s="69"/>
-      <c r="J40" s="69"/>
-      <c r="K40" s="69"/>
-      <c r="L40" s="70"/>
-      <c r="M40" s="71"/>
+      <c r="I40" s="67"/>
+      <c r="J40" s="67"/>
+      <c r="K40" s="67"/>
+      <c r="L40" s="68"/>
+      <c r="M40" s="69"/>
     </row>
     <row r="41" spans="1:13" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="64">
+  <mergeCells count="65">
     <mergeCell ref="B2:C3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="B6:E9"/>
     <mergeCell ref="F6:F9"/>
     <mergeCell ref="G6:G9"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="H6:H9"/>
     <mergeCell ref="I6:I9"/>
     <mergeCell ref="J6:K9"/>

</xml_diff>